<commit_message>
updating the ggplot visualizations
</commit_message>
<xml_diff>
--- a/data/ENVS193_personal_data.xlsx
+++ b/data/ENVS193_personal_data.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="17">
   <si>
     <t>Date (yyyy-mm-dd)</t>
   </si>
@@ -1188,7 +1188,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="13">
-        <v>20.0</v>
+        <v>25.0</v>
       </c>
       <c r="F27" s="11" t="s">
         <v>14</v>
@@ -1649,12 +1649,24 @@
         <f t="shared" si="1"/>
         <v>Thursday</v>
       </c>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
+      <c r="C47" s="18">
+        <v>5.0</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="18">
+        <v>75.0</v>
+      </c>
+      <c r="F47" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="H47" s="18" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="16">
@@ -1664,12 +1676,24 @@
         <f t="shared" si="1"/>
         <v>Friday</v>
       </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
+      <c r="C48" s="18">
+        <v>6.0</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="21">
+        <v>111.0</v>
+      </c>
+      <c r="F48" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="G48" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="H48" s="21" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="16">

</xml_diff>